<commit_message>
Timeline book added to numbers excel file
</commit_message>
<xml_diff>
--- a/docs/numbers.xlsx
+++ b/docs/numbers.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nodir\Projects\open-budget-search\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nodir\Projects\open-budget-search\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{705965E2-B3FE-4DCE-9A07-A68D3CB84289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{101A8129-05E1-4B7C-BAE1-F5A99B42924B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{0AABE945-EFF0-4E0B-A9BD-4BB876D9C82D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{0AABE945-EFF0-4E0B-A9BD-4BB876D9C82D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Timeline" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1420" uniqueCount="1395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1519" uniqueCount="1494">
   <si>
     <t>**-*14-63-61</t>
   </si>
@@ -4219,6 +4220,303 @@
   </si>
   <si>
     <t>**-*70-66-69</t>
+  </si>
+  <si>
+    <t>Country Name</t>
+  </si>
+  <si>
+    <t>12.03.26 10:58</t>
+  </si>
+  <si>
+    <t>13.03.26 17:10</t>
+  </si>
+  <si>
+    <t>15.03.26 06:31</t>
+  </si>
+  <si>
+    <t>15.03.26 19:41</t>
+  </si>
+  <si>
+    <t>15.03.26 21:08</t>
+  </si>
+  <si>
+    <t>16.03.26 05:40</t>
+  </si>
+  <si>
+    <t>16.03.26 09:18</t>
+  </si>
+  <si>
+    <t>16.03.26 11:16</t>
+  </si>
+  <si>
+    <t>16.03.26 15:04</t>
+  </si>
+  <si>
+    <t>16.03.26 17:06</t>
+  </si>
+  <si>
+    <t>16.03.26 18:01</t>
+  </si>
+  <si>
+    <t>16.03.26 20:06</t>
+  </si>
+  <si>
+    <t>17.03.26 09:08</t>
+  </si>
+  <si>
+    <t>17.03.26 09:53</t>
+  </si>
+  <si>
+    <t>17.03.26 10:31</t>
+  </si>
+  <si>
+    <t>17.03.26 11:00</t>
+  </si>
+  <si>
+    <t>17.03.26 11:29</t>
+  </si>
+  <si>
+    <t>17.03.26 11:58</t>
+  </si>
+  <si>
+    <t>17.03.26 12:36</t>
+  </si>
+  <si>
+    <t>17.03.26 13:46</t>
+  </si>
+  <si>
+    <t>17.03.26 14:27</t>
+  </si>
+  <si>
+    <t>17.03.26 14:37</t>
+  </si>
+  <si>
+    <t>17.03.26 15:36</t>
+  </si>
+  <si>
+    <t>17.03.26 15:59</t>
+  </si>
+  <si>
+    <t>17.03.26 16:27</t>
+  </si>
+  <si>
+    <t>17.03.26 16:40</t>
+  </si>
+  <si>
+    <t>17.03.26 17:06</t>
+  </si>
+  <si>
+    <t>17.03.26 17:13</t>
+  </si>
+  <si>
+    <t>17.03.26 17:43</t>
+  </si>
+  <si>
+    <t>17.03.26 19:12</t>
+  </si>
+  <si>
+    <t>17.03.26 22:08</t>
+  </si>
+  <si>
+    <t>17.03.26 22:37</t>
+  </si>
+  <si>
+    <t>17.03.26 23:44</t>
+  </si>
+  <si>
+    <t>18.03.26 06:11</t>
+  </si>
+  <si>
+    <t>18.03.26 09:09</t>
+  </si>
+  <si>
+    <t>18.03.26 09:44</t>
+  </si>
+  <si>
+    <t>18.03.26 10:30</t>
+  </si>
+  <si>
+    <t>18.03.26 11:35</t>
+  </si>
+  <si>
+    <t>18.03.26 12:12</t>
+  </si>
+  <si>
+    <t>18.03.26 12:37</t>
+  </si>
+  <si>
+    <t>18.03.26 13:36</t>
+  </si>
+  <si>
+    <t>18.03.26 15:35</t>
+  </si>
+  <si>
+    <t>18.03.26 17:02</t>
+  </si>
+  <si>
+    <t>18.03.26 18:08</t>
+  </si>
+  <si>
+    <t>18.03.26 20:20</t>
+  </si>
+  <si>
+    <t>18.03.26 23:43</t>
+  </si>
+  <si>
+    <t>19.03.26 01:06</t>
+  </si>
+  <si>
+    <t>19.03.26 08:55</t>
+  </si>
+  <si>
+    <t>19.03.26 10:23</t>
+  </si>
+  <si>
+    <t>19.03.26 10:52</t>
+  </si>
+  <si>
+    <t>19.03.26 11:09</t>
+  </si>
+  <si>
+    <t>19.03.26 12:05</t>
+  </si>
+  <si>
+    <t>19.03.26 12:52</t>
+  </si>
+  <si>
+    <t>19.03.26 13:05</t>
+  </si>
+  <si>
+    <t>19.03.26 13:41</t>
+  </si>
+  <si>
+    <t>19.03.26 14:09</t>
+  </si>
+  <si>
+    <t>19.03.26 14:54</t>
+  </si>
+  <si>
+    <t>19.03.26 15:01</t>
+  </si>
+  <si>
+    <t>19.03.26 16:03</t>
+  </si>
+  <si>
+    <t>19.03.26 16:45</t>
+  </si>
+  <si>
+    <t>19.03.26 17:35</t>
+  </si>
+  <si>
+    <t>19.03.26 22:47</t>
+  </si>
+  <si>
+    <t>19.03.26 23:00</t>
+  </si>
+  <si>
+    <t>19.03.26 23:26</t>
+  </si>
+  <si>
+    <t>20.03.26 01:15</t>
+  </si>
+  <si>
+    <t>20.03.26 02:19</t>
+  </si>
+  <si>
+    <t>20.03.26 08:02</t>
+  </si>
+  <si>
+    <t>20.03.26 08:48</t>
+  </si>
+  <si>
+    <t>20.03.26 13:06</t>
+  </si>
+  <si>
+    <t>20.03.26 13:08</t>
+  </si>
+  <si>
+    <t>20.03.26 13:50</t>
+  </si>
+  <si>
+    <t>20.03.26 14:12</t>
+  </si>
+  <si>
+    <t>20.03.26 14:49</t>
+  </si>
+  <si>
+    <t>20.03.26 15:16</t>
+  </si>
+  <si>
+    <t>20.03.26 15:47</t>
+  </si>
+  <si>
+    <t>20.03.26 16:26</t>
+  </si>
+  <si>
+    <t>20.03.26 16:52</t>
+  </si>
+  <si>
+    <t>20.03.26 19:00</t>
+  </si>
+  <si>
+    <t>20.03.26 19:15</t>
+  </si>
+  <si>
+    <t>20.03.26 19:35</t>
+  </si>
+  <si>
+    <t>20.03.26 19:57</t>
+  </si>
+  <si>
+    <t>20.03.26 20:36</t>
+  </si>
+  <si>
+    <t>20.03.26 21:20</t>
+  </si>
+  <si>
+    <t>20.03.26 21:55</t>
+  </si>
+  <si>
+    <t>20.03.26 22:04</t>
+  </si>
+  <si>
+    <t>20.03.26 23:05</t>
+  </si>
+  <si>
+    <t>20.03.26 23:35</t>
+  </si>
+  <si>
+    <t>20.03.26 23:49</t>
+  </si>
+  <si>
+    <t>20.03.26 23:59</t>
+  </si>
+  <si>
+    <t>Guliston</t>
+  </si>
+  <si>
+    <t>Oydin</t>
+  </si>
+  <si>
+    <t>Qirqquloch</t>
+  </si>
+  <si>
+    <t>Temir yo'l</t>
+  </si>
+  <si>
+    <t>Ko'ksoy</t>
+  </si>
+  <si>
+    <t>Balxiyak</t>
+  </si>
+  <si>
+    <t>Shirinobod</t>
+  </si>
+  <si>
+    <t>Navbahor</t>
+  </si>
+  <si>
+    <t>Ko'ksoy 2</t>
   </si>
 </sst>
 </file>
@@ -19392,4 +19690,2738 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E00F2B87-08AF-4534-8F04-949B3B695D93}">
+  <dimension ref="A2:CL11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="90" width="13.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:90" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1395</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1396</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1397</v>
+      </c>
+      <c r="D2" t="s">
+        <v>1398</v>
+      </c>
+      <c r="E2" t="s">
+        <v>1399</v>
+      </c>
+      <c r="F2" t="s">
+        <v>1400</v>
+      </c>
+      <c r="G2" t="s">
+        <v>1401</v>
+      </c>
+      <c r="H2" t="s">
+        <v>1402</v>
+      </c>
+      <c r="I2" t="s">
+        <v>1403</v>
+      </c>
+      <c r="J2" t="s">
+        <v>1404</v>
+      </c>
+      <c r="K2" t="s">
+        <v>1405</v>
+      </c>
+      <c r="L2" t="s">
+        <v>1406</v>
+      </c>
+      <c r="M2" t="s">
+        <v>1407</v>
+      </c>
+      <c r="N2" t="s">
+        <v>1408</v>
+      </c>
+      <c r="O2" t="s">
+        <v>1409</v>
+      </c>
+      <c r="P2" t="s">
+        <v>1410</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>1411</v>
+      </c>
+      <c r="R2" t="s">
+        <v>1412</v>
+      </c>
+      <c r="S2" t="s">
+        <v>1413</v>
+      </c>
+      <c r="T2" t="s">
+        <v>1414</v>
+      </c>
+      <c r="U2" t="s">
+        <v>1415</v>
+      </c>
+      <c r="V2" t="s">
+        <v>1416</v>
+      </c>
+      <c r="W2" t="s">
+        <v>1417</v>
+      </c>
+      <c r="X2" t="s">
+        <v>1418</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>1419</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>1420</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>1421</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>1422</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>1423</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>1424</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>1425</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>1426</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>1427</v>
+      </c>
+      <c r="AH2" t="s">
+        <v>1428</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>1429</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>1430</v>
+      </c>
+      <c r="AK2" t="s">
+        <v>1431</v>
+      </c>
+      <c r="AL2" t="s">
+        <v>1432</v>
+      </c>
+      <c r="AM2" t="s">
+        <v>1433</v>
+      </c>
+      <c r="AN2" t="s">
+        <v>1434</v>
+      </c>
+      <c r="AO2" t="s">
+        <v>1435</v>
+      </c>
+      <c r="AP2" t="s">
+        <v>1436</v>
+      </c>
+      <c r="AQ2" t="s">
+        <v>1437</v>
+      </c>
+      <c r="AR2" t="s">
+        <v>1438</v>
+      </c>
+      <c r="AS2" t="s">
+        <v>1439</v>
+      </c>
+      <c r="AT2" t="s">
+        <v>1440</v>
+      </c>
+      <c r="AU2" t="s">
+        <v>1441</v>
+      </c>
+      <c r="AV2" t="s">
+        <v>1442</v>
+      </c>
+      <c r="AW2" t="s">
+        <v>1443</v>
+      </c>
+      <c r="AX2" t="s">
+        <v>1444</v>
+      </c>
+      <c r="AY2" t="s">
+        <v>1445</v>
+      </c>
+      <c r="AZ2" t="s">
+        <v>1446</v>
+      </c>
+      <c r="BA2" t="s">
+        <v>1447</v>
+      </c>
+      <c r="BB2" t="s">
+        <v>1448</v>
+      </c>
+      <c r="BC2" t="s">
+        <v>1449</v>
+      </c>
+      <c r="BD2" t="s">
+        <v>1450</v>
+      </c>
+      <c r="BE2" t="s">
+        <v>1451</v>
+      </c>
+      <c r="BF2" t="s">
+        <v>1452</v>
+      </c>
+      <c r="BG2" t="s">
+        <v>1453</v>
+      </c>
+      <c r="BH2" t="s">
+        <v>1454</v>
+      </c>
+      <c r="BI2" t="s">
+        <v>1455</v>
+      </c>
+      <c r="BJ2" t="s">
+        <v>1456</v>
+      </c>
+      <c r="BK2" t="s">
+        <v>1457</v>
+      </c>
+      <c r="BL2" t="s">
+        <v>1458</v>
+      </c>
+      <c r="BM2" t="s">
+        <v>1459</v>
+      </c>
+      <c r="BN2" t="s">
+        <v>1460</v>
+      </c>
+      <c r="BO2" t="s">
+        <v>1461</v>
+      </c>
+      <c r="BP2" t="s">
+        <v>1462</v>
+      </c>
+      <c r="BQ2" t="s">
+        <v>1463</v>
+      </c>
+      <c r="BR2" t="s">
+        <v>1464</v>
+      </c>
+      <c r="BS2" t="s">
+        <v>1465</v>
+      </c>
+      <c r="BT2" t="s">
+        <v>1466</v>
+      </c>
+      <c r="BU2" t="s">
+        <v>1467</v>
+      </c>
+      <c r="BV2" t="s">
+        <v>1468</v>
+      </c>
+      <c r="BW2" t="s">
+        <v>1469</v>
+      </c>
+      <c r="BX2" t="s">
+        <v>1470</v>
+      </c>
+      <c r="BY2" t="s">
+        <v>1471</v>
+      </c>
+      <c r="BZ2" t="s">
+        <v>1472</v>
+      </c>
+      <c r="CA2" t="s">
+        <v>1473</v>
+      </c>
+      <c r="CB2" t="s">
+        <v>1474</v>
+      </c>
+      <c r="CC2" t="s">
+        <v>1475</v>
+      </c>
+      <c r="CD2" t="s">
+        <v>1476</v>
+      </c>
+      <c r="CE2" t="s">
+        <v>1477</v>
+      </c>
+      <c r="CF2" t="s">
+        <v>1478</v>
+      </c>
+      <c r="CG2" t="s">
+        <v>1479</v>
+      </c>
+      <c r="CH2" t="s">
+        <v>1480</v>
+      </c>
+      <c r="CI2" t="s">
+        <v>1481</v>
+      </c>
+      <c r="CJ2" t="s">
+        <v>1482</v>
+      </c>
+      <c r="CK2" t="s">
+        <v>1483</v>
+      </c>
+      <c r="CL2" t="s">
+        <v>1484</v>
+      </c>
+    </row>
+    <row r="3" spans="1:90" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>1485</v>
+      </c>
+      <c r="B3">
+        <v>759</v>
+      </c>
+      <c r="C3">
+        <v>1385</v>
+      </c>
+      <c r="D3">
+        <v>3041</v>
+      </c>
+      <c r="E3">
+        <v>4052</v>
+      </c>
+      <c r="F3">
+        <v>4076</v>
+      </c>
+      <c r="G3">
+        <v>4174</v>
+      </c>
+      <c r="H3">
+        <v>4209</v>
+      </c>
+      <c r="I3">
+        <v>4319</v>
+      </c>
+      <c r="J3">
+        <v>4684</v>
+      </c>
+      <c r="K3">
+        <v>4797</v>
+      </c>
+      <c r="L3">
+        <v>4914</v>
+      </c>
+      <c r="M3">
+        <v>4990</v>
+      </c>
+      <c r="N3">
+        <v>5153</v>
+      </c>
+      <c r="O3">
+        <v>5188</v>
+      </c>
+      <c r="P3">
+        <v>5203</v>
+      </c>
+      <c r="Q3">
+        <v>5222</v>
+      </c>
+      <c r="R3">
+        <v>5241</v>
+      </c>
+      <c r="S3">
+        <v>5268</v>
+      </c>
+      <c r="T3">
+        <v>5324</v>
+      </c>
+      <c r="U3">
+        <v>5479</v>
+      </c>
+      <c r="V3">
+        <v>5568</v>
+      </c>
+      <c r="W3">
+        <v>5668</v>
+      </c>
+      <c r="X3">
+        <v>5784</v>
+      </c>
+      <c r="Y3">
+        <v>5872</v>
+      </c>
+      <c r="Z3">
+        <v>5914</v>
+      </c>
+      <c r="AA3">
+        <v>5964</v>
+      </c>
+      <c r="AB3">
+        <v>5964</v>
+      </c>
+      <c r="AC3">
+        <v>6005</v>
+      </c>
+      <c r="AD3">
+        <v>6040</v>
+      </c>
+      <c r="AE3">
+        <v>6113</v>
+      </c>
+      <c r="AF3">
+        <v>6226</v>
+      </c>
+      <c r="AG3">
+        <v>6228</v>
+      </c>
+      <c r="AH3">
+        <v>6255</v>
+      </c>
+      <c r="AI3">
+        <v>6377</v>
+      </c>
+      <c r="AJ3">
+        <v>6383</v>
+      </c>
+      <c r="AK3">
+        <v>6384</v>
+      </c>
+      <c r="AL3">
+        <v>6402</v>
+      </c>
+      <c r="AM3">
+        <v>6494</v>
+      </c>
+      <c r="AN3">
+        <v>6540</v>
+      </c>
+      <c r="AO3">
+        <v>6570</v>
+      </c>
+      <c r="AP3">
+        <v>6613</v>
+      </c>
+      <c r="AQ3">
+        <v>6734</v>
+      </c>
+      <c r="AR3">
+        <v>6778</v>
+      </c>
+      <c r="AS3">
+        <v>6854</v>
+      </c>
+      <c r="AT3">
+        <v>6964</v>
+      </c>
+      <c r="AU3">
+        <v>7172</v>
+      </c>
+      <c r="AV3">
+        <v>7217</v>
+      </c>
+      <c r="AW3">
+        <v>7253</v>
+      </c>
+      <c r="AX3">
+        <v>7324</v>
+      </c>
+      <c r="AY3">
+        <v>7355</v>
+      </c>
+      <c r="AZ3">
+        <v>7446</v>
+      </c>
+      <c r="BA3">
+        <v>7666</v>
+      </c>
+      <c r="BB3">
+        <v>7812</v>
+      </c>
+      <c r="BC3">
+        <v>8038</v>
+      </c>
+      <c r="BD3">
+        <v>8191</v>
+      </c>
+      <c r="BE3">
+        <v>8328</v>
+      </c>
+      <c r="BF3">
+        <v>8384</v>
+      </c>
+      <c r="BG3">
+        <v>8444</v>
+      </c>
+      <c r="BH3">
+        <v>8481</v>
+      </c>
+      <c r="BI3">
+        <v>8585</v>
+      </c>
+      <c r="BJ3">
+        <v>8642</v>
+      </c>
+      <c r="BK3">
+        <v>8976</v>
+      </c>
+      <c r="BL3">
+        <v>8984</v>
+      </c>
+      <c r="BM3">
+        <v>8990</v>
+      </c>
+      <c r="BN3">
+        <v>9064</v>
+      </c>
+      <c r="BO3">
+        <v>9172</v>
+      </c>
+      <c r="BP3">
+        <v>9234</v>
+      </c>
+      <c r="BQ3">
+        <v>9234</v>
+      </c>
+      <c r="BR3">
+        <v>9385</v>
+      </c>
+      <c r="BS3">
+        <v>9473</v>
+      </c>
+      <c r="BT3">
+        <v>9559</v>
+      </c>
+      <c r="BU3">
+        <v>9637</v>
+      </c>
+      <c r="BV3">
+        <v>9696</v>
+      </c>
+      <c r="BW3">
+        <v>9794</v>
+      </c>
+      <c r="BX3">
+        <v>9941</v>
+      </c>
+      <c r="BY3">
+        <v>10198</v>
+      </c>
+      <c r="BZ3">
+        <v>10397</v>
+      </c>
+      <c r="CA3">
+        <v>11002</v>
+      </c>
+      <c r="CB3">
+        <v>11205</v>
+      </c>
+      <c r="CC3">
+        <v>11332</v>
+      </c>
+      <c r="CD3">
+        <v>11426</v>
+      </c>
+      <c r="CE3">
+        <v>11515</v>
+      </c>
+      <c r="CF3">
+        <v>11586</v>
+      </c>
+      <c r="CG3">
+        <v>11688</v>
+      </c>
+      <c r="CH3">
+        <v>11790</v>
+      </c>
+      <c r="CI3">
+        <v>12060</v>
+      </c>
+      <c r="CJ3">
+        <v>12131</v>
+      </c>
+      <c r="CK3">
+        <v>12294</v>
+      </c>
+      <c r="CL3">
+        <v>12297</v>
+      </c>
+    </row>
+    <row r="4" spans="1:90" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>1486</v>
+      </c>
+      <c r="B4">
+        <v>840</v>
+      </c>
+      <c r="C4">
+        <v>1822</v>
+      </c>
+      <c r="D4">
+        <v>2903</v>
+      </c>
+      <c r="E4">
+        <v>3808</v>
+      </c>
+      <c r="F4">
+        <v>3860</v>
+      </c>
+      <c r="G4">
+        <v>3968</v>
+      </c>
+      <c r="H4">
+        <v>3985</v>
+      </c>
+      <c r="I4">
+        <v>4152</v>
+      </c>
+      <c r="J4">
+        <v>4654</v>
+      </c>
+      <c r="K4">
+        <v>4839</v>
+      </c>
+      <c r="L4">
+        <v>5011</v>
+      </c>
+      <c r="M4">
+        <v>5174</v>
+      </c>
+      <c r="N4">
+        <v>5392</v>
+      </c>
+      <c r="O4">
+        <v>5405</v>
+      </c>
+      <c r="P4">
+        <v>5427</v>
+      </c>
+      <c r="Q4">
+        <v>5471</v>
+      </c>
+      <c r="R4">
+        <v>5513</v>
+      </c>
+      <c r="S4">
+        <v>5586</v>
+      </c>
+      <c r="T4">
+        <v>5675</v>
+      </c>
+      <c r="U4">
+        <v>5888</v>
+      </c>
+      <c r="V4">
+        <v>6007</v>
+      </c>
+      <c r="W4">
+        <v>6097</v>
+      </c>
+      <c r="X4">
+        <v>6182</v>
+      </c>
+      <c r="Y4">
+        <v>6272</v>
+      </c>
+      <c r="Z4">
+        <v>6339</v>
+      </c>
+      <c r="AA4">
+        <v>6360</v>
+      </c>
+      <c r="AB4">
+        <v>6360</v>
+      </c>
+      <c r="AC4">
+        <v>6384</v>
+      </c>
+      <c r="AD4">
+        <v>6434</v>
+      </c>
+      <c r="AE4">
+        <v>6477</v>
+      </c>
+      <c r="AF4">
+        <v>6526</v>
+      </c>
+      <c r="AG4">
+        <v>6542</v>
+      </c>
+      <c r="AH4">
+        <v>6566</v>
+      </c>
+      <c r="AI4">
+        <v>6582</v>
+      </c>
+      <c r="AJ4">
+        <v>6588</v>
+      </c>
+      <c r="AK4">
+        <v>6591</v>
+      </c>
+      <c r="AL4">
+        <v>6649</v>
+      </c>
+      <c r="AM4">
+        <v>6851</v>
+      </c>
+      <c r="AN4">
+        <v>6956</v>
+      </c>
+      <c r="AO4">
+        <v>7103</v>
+      </c>
+      <c r="AP4">
+        <v>7262</v>
+      </c>
+      <c r="AQ4">
+        <v>7505</v>
+      </c>
+      <c r="AR4">
+        <v>7639</v>
+      </c>
+      <c r="AS4">
+        <v>7793</v>
+      </c>
+      <c r="AT4">
+        <v>7909</v>
+      </c>
+      <c r="AU4">
+        <v>7939</v>
+      </c>
+      <c r="AV4">
+        <v>7940</v>
+      </c>
+      <c r="AW4">
+        <v>7947</v>
+      </c>
+      <c r="AX4">
+        <v>7954</v>
+      </c>
+      <c r="AY4">
+        <v>7986</v>
+      </c>
+      <c r="AZ4">
+        <v>8021</v>
+      </c>
+      <c r="BA4">
+        <v>8182</v>
+      </c>
+      <c r="BB4">
+        <v>8303</v>
+      </c>
+      <c r="BC4">
+        <v>8447</v>
+      </c>
+      <c r="BD4">
+        <v>8548</v>
+      </c>
+      <c r="BE4">
+        <v>8641</v>
+      </c>
+      <c r="BF4">
+        <v>8686</v>
+      </c>
+      <c r="BG4">
+        <v>8743</v>
+      </c>
+      <c r="BH4">
+        <v>8812</v>
+      </c>
+      <c r="BI4">
+        <v>8931</v>
+      </c>
+      <c r="BJ4">
+        <v>8974</v>
+      </c>
+      <c r="BK4">
+        <v>9272</v>
+      </c>
+      <c r="BL4">
+        <v>9299</v>
+      </c>
+      <c r="BM4">
+        <v>9319</v>
+      </c>
+      <c r="BN4">
+        <v>9419</v>
+      </c>
+      <c r="BO4">
+        <v>9420</v>
+      </c>
+      <c r="BP4">
+        <v>9421</v>
+      </c>
+      <c r="BQ4">
+        <v>9422</v>
+      </c>
+      <c r="BR4">
+        <v>9761</v>
+      </c>
+      <c r="BS4">
+        <v>9894</v>
+      </c>
+      <c r="BT4">
+        <v>9975</v>
+      </c>
+      <c r="BU4">
+        <v>10089</v>
+      </c>
+      <c r="BV4">
+        <v>10172</v>
+      </c>
+      <c r="BW4">
+        <v>10271</v>
+      </c>
+      <c r="BX4">
+        <v>10342</v>
+      </c>
+      <c r="BY4">
+        <v>10444</v>
+      </c>
+      <c r="BZ4">
+        <v>10543</v>
+      </c>
+      <c r="CA4">
+        <v>10816</v>
+      </c>
+      <c r="CB4">
+        <v>10944</v>
+      </c>
+      <c r="CC4">
+        <v>11094</v>
+      </c>
+      <c r="CD4">
+        <v>11246</v>
+      </c>
+      <c r="CE4">
+        <v>11346</v>
+      </c>
+      <c r="CF4">
+        <v>11482</v>
+      </c>
+      <c r="CG4">
+        <v>11626</v>
+      </c>
+      <c r="CH4">
+        <v>11718</v>
+      </c>
+      <c r="CI4">
+        <v>12136</v>
+      </c>
+      <c r="CJ4">
+        <v>12150</v>
+      </c>
+      <c r="CK4">
+        <v>12269</v>
+      </c>
+      <c r="CL4">
+        <v>12270</v>
+      </c>
+    </row>
+    <row r="5" spans="1:90" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>1487</v>
+      </c>
+      <c r="B5">
+        <v>679</v>
+      </c>
+      <c r="C5">
+        <v>1465</v>
+      </c>
+      <c r="D5">
+        <v>2751</v>
+      </c>
+      <c r="E5">
+        <v>3838</v>
+      </c>
+      <c r="F5">
+        <v>3873</v>
+      </c>
+      <c r="G5">
+        <v>3929</v>
+      </c>
+      <c r="H5">
+        <v>3930</v>
+      </c>
+      <c r="I5">
+        <v>4145</v>
+      </c>
+      <c r="J5">
+        <v>4486</v>
+      </c>
+      <c r="K5">
+        <v>4544</v>
+      </c>
+      <c r="L5">
+        <v>4613</v>
+      </c>
+      <c r="M5">
+        <v>4676</v>
+      </c>
+      <c r="N5">
+        <v>4733</v>
+      </c>
+      <c r="O5">
+        <v>4769</v>
+      </c>
+      <c r="P5">
+        <v>4809</v>
+      </c>
+      <c r="Q5">
+        <v>4863</v>
+      </c>
+      <c r="R5">
+        <v>4913</v>
+      </c>
+      <c r="S5">
+        <v>5013</v>
+      </c>
+      <c r="T5">
+        <v>5057</v>
+      </c>
+      <c r="U5">
+        <v>5154</v>
+      </c>
+      <c r="V5">
+        <v>5195</v>
+      </c>
+      <c r="W5">
+        <v>5243</v>
+      </c>
+      <c r="X5">
+        <v>5291</v>
+      </c>
+      <c r="Y5">
+        <v>5333</v>
+      </c>
+      <c r="Z5">
+        <v>5395</v>
+      </c>
+      <c r="AA5">
+        <v>5433</v>
+      </c>
+      <c r="AB5">
+        <v>5433</v>
+      </c>
+      <c r="AC5">
+        <v>5442</v>
+      </c>
+      <c r="AD5">
+        <v>5444</v>
+      </c>
+      <c r="AE5">
+        <v>5474</v>
+      </c>
+      <c r="AF5">
+        <v>5542</v>
+      </c>
+      <c r="AG5">
+        <v>5571</v>
+      </c>
+      <c r="AH5">
+        <v>5623</v>
+      </c>
+      <c r="AI5">
+        <v>5654</v>
+      </c>
+      <c r="AJ5">
+        <v>5658</v>
+      </c>
+      <c r="AK5">
+        <v>5660</v>
+      </c>
+      <c r="AL5">
+        <v>5688</v>
+      </c>
+      <c r="AM5">
+        <v>5818</v>
+      </c>
+      <c r="AN5">
+        <v>5879</v>
+      </c>
+      <c r="AO5">
+        <v>5954</v>
+      </c>
+      <c r="AP5">
+        <v>6016</v>
+      </c>
+      <c r="AQ5">
+        <v>6079</v>
+      </c>
+      <c r="AR5">
+        <v>6199</v>
+      </c>
+      <c r="AS5">
+        <v>6258</v>
+      </c>
+      <c r="AT5">
+        <v>6287</v>
+      </c>
+      <c r="AU5">
+        <v>6411</v>
+      </c>
+      <c r="AV5">
+        <v>6421</v>
+      </c>
+      <c r="AW5">
+        <v>6582</v>
+      </c>
+      <c r="AX5">
+        <v>6588</v>
+      </c>
+      <c r="AY5">
+        <v>6595</v>
+      </c>
+      <c r="AZ5">
+        <v>6625</v>
+      </c>
+      <c r="BA5">
+        <v>6715</v>
+      </c>
+      <c r="BB5">
+        <v>6812</v>
+      </c>
+      <c r="BC5">
+        <v>6954</v>
+      </c>
+      <c r="BD5">
+        <v>7102</v>
+      </c>
+      <c r="BE5">
+        <v>7232</v>
+      </c>
+      <c r="BF5">
+        <v>7377</v>
+      </c>
+      <c r="BG5">
+        <v>7520</v>
+      </c>
+      <c r="BH5">
+        <v>7640</v>
+      </c>
+      <c r="BI5">
+        <v>7844</v>
+      </c>
+      <c r="BJ5">
+        <v>7987</v>
+      </c>
+      <c r="BK5">
+        <v>8740</v>
+      </c>
+      <c r="BL5">
+        <v>8792</v>
+      </c>
+      <c r="BM5">
+        <v>8845</v>
+      </c>
+      <c r="BN5">
+        <v>8972</v>
+      </c>
+      <c r="BO5">
+        <v>8972</v>
+      </c>
+      <c r="BP5">
+        <v>8978</v>
+      </c>
+      <c r="BQ5">
+        <v>8982</v>
+      </c>
+      <c r="BR5">
+        <v>9640</v>
+      </c>
+      <c r="BS5">
+        <v>9724</v>
+      </c>
+      <c r="BT5">
+        <v>9816</v>
+      </c>
+      <c r="BU5">
+        <v>9897</v>
+      </c>
+      <c r="BV5">
+        <v>10008</v>
+      </c>
+      <c r="BW5">
+        <v>10110</v>
+      </c>
+      <c r="BX5">
+        <v>10200</v>
+      </c>
+      <c r="BY5">
+        <v>10305</v>
+      </c>
+      <c r="BZ5">
+        <v>10412</v>
+      </c>
+      <c r="CA5">
+        <v>10850</v>
+      </c>
+      <c r="CB5">
+        <v>10950</v>
+      </c>
+      <c r="CC5">
+        <v>11073</v>
+      </c>
+      <c r="CD5">
+        <v>11181</v>
+      </c>
+      <c r="CE5">
+        <v>11277</v>
+      </c>
+      <c r="CF5">
+        <v>11374</v>
+      </c>
+      <c r="CG5">
+        <v>11444</v>
+      </c>
+      <c r="CH5">
+        <v>11541</v>
+      </c>
+      <c r="CI5">
+        <v>11851</v>
+      </c>
+      <c r="CJ5">
+        <v>11920</v>
+      </c>
+      <c r="CK5">
+        <v>11993</v>
+      </c>
+      <c r="CL5">
+        <v>11993</v>
+      </c>
+    </row>
+    <row r="6" spans="1:90" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>1488</v>
+      </c>
+      <c r="B6">
+        <v>1722</v>
+      </c>
+      <c r="C6">
+        <v>3075</v>
+      </c>
+      <c r="D6">
+        <v>3867</v>
+      </c>
+      <c r="E6">
+        <v>4380</v>
+      </c>
+      <c r="F6">
+        <v>4405</v>
+      </c>
+      <c r="G6">
+        <v>4427</v>
+      </c>
+      <c r="H6">
+        <v>4428</v>
+      </c>
+      <c r="I6">
+        <v>4454</v>
+      </c>
+      <c r="J6">
+        <v>4632</v>
+      </c>
+      <c r="K6">
+        <v>4693</v>
+      </c>
+      <c r="L6">
+        <v>4729</v>
+      </c>
+      <c r="M6">
+        <v>4744</v>
+      </c>
+      <c r="N6">
+        <v>4789</v>
+      </c>
+      <c r="O6">
+        <v>4791</v>
+      </c>
+      <c r="P6">
+        <v>4794</v>
+      </c>
+      <c r="Q6">
+        <v>4846</v>
+      </c>
+      <c r="R6">
+        <v>4892</v>
+      </c>
+      <c r="S6">
+        <v>4961</v>
+      </c>
+      <c r="T6">
+        <v>5045</v>
+      </c>
+      <c r="U6">
+        <v>5139</v>
+      </c>
+      <c r="V6">
+        <v>5186</v>
+      </c>
+      <c r="W6">
+        <v>5246</v>
+      </c>
+      <c r="X6">
+        <v>5281</v>
+      </c>
+      <c r="Y6">
+        <v>5325</v>
+      </c>
+      <c r="Z6">
+        <v>5378</v>
+      </c>
+      <c r="AA6">
+        <v>5427</v>
+      </c>
+      <c r="AB6">
+        <v>5427</v>
+      </c>
+      <c r="AC6">
+        <v>5487</v>
+      </c>
+      <c r="AD6">
+        <v>5540</v>
+      </c>
+      <c r="AE6">
+        <v>5576</v>
+      </c>
+      <c r="AF6">
+        <v>5694</v>
+      </c>
+      <c r="AG6">
+        <v>5700</v>
+      </c>
+      <c r="AH6">
+        <v>5724</v>
+      </c>
+      <c r="AI6">
+        <v>5769</v>
+      </c>
+      <c r="AJ6">
+        <v>5770</v>
+      </c>
+      <c r="AK6">
+        <v>5771</v>
+      </c>
+      <c r="AL6">
+        <v>5780</v>
+      </c>
+      <c r="AM6">
+        <v>5803</v>
+      </c>
+      <c r="AN6">
+        <v>5836</v>
+      </c>
+      <c r="AO6">
+        <v>5866</v>
+      </c>
+      <c r="AP6">
+        <v>5911</v>
+      </c>
+      <c r="AQ6">
+        <v>6044</v>
+      </c>
+      <c r="AR6">
+        <v>6163</v>
+      </c>
+      <c r="AS6">
+        <v>6182</v>
+      </c>
+      <c r="AT6">
+        <v>6277</v>
+      </c>
+      <c r="AU6">
+        <v>6572</v>
+      </c>
+      <c r="AV6">
+        <v>6594</v>
+      </c>
+      <c r="AW6">
+        <v>6601</v>
+      </c>
+      <c r="AX6">
+        <v>6607</v>
+      </c>
+      <c r="AY6">
+        <v>6608</v>
+      </c>
+      <c r="AZ6">
+        <v>6624</v>
+      </c>
+      <c r="BA6">
+        <v>6648</v>
+      </c>
+      <c r="BB6">
+        <v>6658</v>
+      </c>
+      <c r="BC6">
+        <v>6665</v>
+      </c>
+      <c r="BD6">
+        <v>6680</v>
+      </c>
+      <c r="BE6">
+        <v>6695</v>
+      </c>
+      <c r="BF6">
+        <v>6708</v>
+      </c>
+      <c r="BG6">
+        <v>6723</v>
+      </c>
+      <c r="BH6">
+        <v>6810</v>
+      </c>
+      <c r="BI6">
+        <v>7003</v>
+      </c>
+      <c r="BJ6">
+        <v>7069</v>
+      </c>
+      <c r="BK6">
+        <v>7637</v>
+      </c>
+      <c r="BL6">
+        <v>7652</v>
+      </c>
+      <c r="BM6">
+        <v>7683</v>
+      </c>
+      <c r="BN6">
+        <v>7710</v>
+      </c>
+      <c r="BO6">
+        <v>7824</v>
+      </c>
+      <c r="BP6">
+        <v>7869</v>
+      </c>
+      <c r="BQ6">
+        <v>7870</v>
+      </c>
+      <c r="BR6">
+        <v>7889</v>
+      </c>
+      <c r="BS6">
+        <v>7892</v>
+      </c>
+      <c r="BT6">
+        <v>7909</v>
+      </c>
+      <c r="BU6">
+        <v>7989</v>
+      </c>
+      <c r="BV6">
+        <v>8126</v>
+      </c>
+      <c r="BW6">
+        <v>8323</v>
+      </c>
+      <c r="BX6">
+        <v>8552</v>
+      </c>
+      <c r="BY6">
+        <v>8799</v>
+      </c>
+      <c r="BZ6">
+        <v>8984</v>
+      </c>
+      <c r="CA6">
+        <v>9357</v>
+      </c>
+      <c r="CB6">
+        <v>9497</v>
+      </c>
+      <c r="CC6">
+        <v>9676</v>
+      </c>
+      <c r="CD6">
+        <v>9863</v>
+      </c>
+      <c r="CE6">
+        <v>10035</v>
+      </c>
+      <c r="CF6">
+        <v>10313</v>
+      </c>
+      <c r="CG6">
+        <v>10672</v>
+      </c>
+      <c r="CH6">
+        <v>10984</v>
+      </c>
+      <c r="CI6">
+        <v>11799</v>
+      </c>
+      <c r="CJ6">
+        <v>11851</v>
+      </c>
+      <c r="CK6">
+        <v>11886</v>
+      </c>
+      <c r="CL6">
+        <v>11886</v>
+      </c>
+    </row>
+    <row r="7" spans="1:90" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>1489</v>
+      </c>
+      <c r="B7">
+        <v>1477</v>
+      </c>
+      <c r="C7">
+        <v>2787</v>
+      </c>
+      <c r="D7">
+        <v>3662</v>
+      </c>
+      <c r="E7">
+        <v>4267</v>
+      </c>
+      <c r="F7">
+        <v>4272</v>
+      </c>
+      <c r="G7">
+        <v>4233</v>
+      </c>
+      <c r="H7">
+        <v>4235</v>
+      </c>
+      <c r="I7">
+        <v>4296</v>
+      </c>
+      <c r="J7">
+        <v>4563</v>
+      </c>
+      <c r="K7">
+        <v>4662</v>
+      </c>
+      <c r="L7">
+        <v>4822</v>
+      </c>
+      <c r="M7">
+        <v>5056</v>
+      </c>
+      <c r="N7">
+        <v>5320</v>
+      </c>
+      <c r="O7">
+        <v>5357</v>
+      </c>
+      <c r="P7">
+        <v>5416</v>
+      </c>
+      <c r="Q7">
+        <v>5484</v>
+      </c>
+      <c r="R7">
+        <v>5556</v>
+      </c>
+      <c r="S7">
+        <v>5629</v>
+      </c>
+      <c r="T7">
+        <v>5682</v>
+      </c>
+      <c r="U7">
+        <v>5772</v>
+      </c>
+      <c r="V7">
+        <v>5818</v>
+      </c>
+      <c r="W7">
+        <v>5843</v>
+      </c>
+      <c r="X7">
+        <v>5875</v>
+      </c>
+      <c r="Y7">
+        <v>5917</v>
+      </c>
+      <c r="Z7">
+        <v>5970</v>
+      </c>
+      <c r="AA7">
+        <v>6047</v>
+      </c>
+      <c r="AB7">
+        <v>6047</v>
+      </c>
+      <c r="AC7">
+        <v>6150</v>
+      </c>
+      <c r="AD7">
+        <v>6219</v>
+      </c>
+      <c r="AE7">
+        <v>6328</v>
+      </c>
+      <c r="AF7">
+        <v>6534</v>
+      </c>
+      <c r="AG7">
+        <v>6538</v>
+      </c>
+      <c r="AH7">
+        <v>6541</v>
+      </c>
+      <c r="AI7">
+        <v>6596</v>
+      </c>
+      <c r="AJ7">
+        <v>6598</v>
+      </c>
+      <c r="AK7">
+        <v>6598</v>
+      </c>
+      <c r="AL7">
+        <v>6629</v>
+      </c>
+      <c r="AM7">
+        <v>6688</v>
+      </c>
+      <c r="AN7">
+        <v>6721</v>
+      </c>
+      <c r="AO7">
+        <v>6772</v>
+      </c>
+      <c r="AP7">
+        <v>6822</v>
+      </c>
+      <c r="AQ7">
+        <v>6934</v>
+      </c>
+      <c r="AR7">
+        <v>6980</v>
+      </c>
+      <c r="AS7">
+        <v>7059</v>
+      </c>
+      <c r="AT7">
+        <v>7105</v>
+      </c>
+      <c r="AU7">
+        <v>7136</v>
+      </c>
+      <c r="AV7">
+        <v>7138</v>
+      </c>
+      <c r="AW7">
+        <v>7166</v>
+      </c>
+      <c r="AX7">
+        <v>7186</v>
+      </c>
+      <c r="AY7">
+        <v>7205</v>
+      </c>
+      <c r="AZ7">
+        <v>7236</v>
+      </c>
+      <c r="BA7">
+        <v>7345</v>
+      </c>
+      <c r="BB7">
+        <v>7403</v>
+      </c>
+      <c r="BC7">
+        <v>7496</v>
+      </c>
+      <c r="BD7">
+        <v>7613</v>
+      </c>
+      <c r="BE7">
+        <v>7730</v>
+      </c>
+      <c r="BF7">
+        <v>7848</v>
+      </c>
+      <c r="BG7">
+        <v>7960</v>
+      </c>
+      <c r="BH7">
+        <v>8076</v>
+      </c>
+      <c r="BI7">
+        <v>8318</v>
+      </c>
+      <c r="BJ7">
+        <v>8441</v>
+      </c>
+      <c r="BK7">
+        <v>9001</v>
+      </c>
+      <c r="BL7">
+        <v>9042</v>
+      </c>
+      <c r="BM7">
+        <v>9102</v>
+      </c>
+      <c r="BN7">
+        <v>9135</v>
+      </c>
+      <c r="BO7">
+        <v>9135</v>
+      </c>
+      <c r="BP7">
+        <v>9137</v>
+      </c>
+      <c r="BQ7">
+        <v>9137</v>
+      </c>
+      <c r="BR7">
+        <v>9472</v>
+      </c>
+      <c r="BS7">
+        <v>9549</v>
+      </c>
+      <c r="BT7">
+        <v>9637</v>
+      </c>
+      <c r="BU7">
+        <v>9694</v>
+      </c>
+      <c r="BV7">
+        <v>9722</v>
+      </c>
+      <c r="BW7">
+        <v>9766</v>
+      </c>
+      <c r="BX7">
+        <v>9829</v>
+      </c>
+      <c r="BY7">
+        <v>9882</v>
+      </c>
+      <c r="BZ7">
+        <v>9935</v>
+      </c>
+      <c r="CA7">
+        <v>10274</v>
+      </c>
+      <c r="CB7">
+        <v>10425</v>
+      </c>
+      <c r="CC7">
+        <v>10560</v>
+      </c>
+      <c r="CD7">
+        <v>10726</v>
+      </c>
+      <c r="CE7">
+        <v>10920</v>
+      </c>
+      <c r="CF7">
+        <v>11099</v>
+      </c>
+      <c r="CG7">
+        <v>11243</v>
+      </c>
+      <c r="CH7">
+        <v>11357</v>
+      </c>
+      <c r="CI7">
+        <v>11626</v>
+      </c>
+      <c r="CJ7">
+        <v>11685</v>
+      </c>
+      <c r="CK7">
+        <v>11719</v>
+      </c>
+      <c r="CL7">
+        <v>11720</v>
+      </c>
+    </row>
+    <row r="8" spans="1:90" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>1490</v>
+      </c>
+      <c r="B8">
+        <v>1859</v>
+      </c>
+      <c r="C8">
+        <v>3803</v>
+      </c>
+      <c r="D8">
+        <v>4789</v>
+      </c>
+      <c r="E8">
+        <v>5278</v>
+      </c>
+      <c r="F8">
+        <v>5290</v>
+      </c>
+      <c r="G8">
+        <v>5273</v>
+      </c>
+      <c r="H8">
+        <v>5275</v>
+      </c>
+      <c r="I8">
+        <v>5290</v>
+      </c>
+      <c r="J8">
+        <v>5433</v>
+      </c>
+      <c r="K8">
+        <v>5504</v>
+      </c>
+      <c r="L8">
+        <v>5538</v>
+      </c>
+      <c r="M8">
+        <v>5543</v>
+      </c>
+      <c r="N8">
+        <v>5621</v>
+      </c>
+      <c r="O8">
+        <v>5780</v>
+      </c>
+      <c r="P8">
+        <v>5866</v>
+      </c>
+      <c r="Q8">
+        <v>5968</v>
+      </c>
+      <c r="R8">
+        <v>6044</v>
+      </c>
+      <c r="S8">
+        <v>6125</v>
+      </c>
+      <c r="T8">
+        <v>6225</v>
+      </c>
+      <c r="U8">
+        <v>6334</v>
+      </c>
+      <c r="V8">
+        <v>6365</v>
+      </c>
+      <c r="W8">
+        <v>6385</v>
+      </c>
+      <c r="X8">
+        <v>6388</v>
+      </c>
+      <c r="Y8">
+        <v>6388</v>
+      </c>
+      <c r="Z8">
+        <v>6393</v>
+      </c>
+      <c r="AA8">
+        <v>6400</v>
+      </c>
+      <c r="AB8">
+        <v>6400</v>
+      </c>
+      <c r="AC8">
+        <v>6452</v>
+      </c>
+      <c r="AD8">
+        <v>6472</v>
+      </c>
+      <c r="AE8">
+        <v>6515</v>
+      </c>
+      <c r="AF8">
+        <v>6603</v>
+      </c>
+      <c r="AG8">
+        <v>6613</v>
+      </c>
+      <c r="AH8">
+        <v>6629</v>
+      </c>
+      <c r="AI8">
+        <v>6681</v>
+      </c>
+      <c r="AJ8">
+        <v>6685</v>
+      </c>
+      <c r="AK8">
+        <v>6693</v>
+      </c>
+      <c r="AL8">
+        <v>6720</v>
+      </c>
+      <c r="AM8">
+        <v>6809</v>
+      </c>
+      <c r="AN8">
+        <v>6890</v>
+      </c>
+      <c r="AO8">
+        <v>6972</v>
+      </c>
+      <c r="AP8">
+        <v>7081</v>
+      </c>
+      <c r="AQ8">
+        <v>7278</v>
+      </c>
+      <c r="AR8">
+        <v>7540</v>
+      </c>
+      <c r="AS8">
+        <v>7585</v>
+      </c>
+      <c r="AT8">
+        <v>7654</v>
+      </c>
+      <c r="AU8">
+        <v>7715</v>
+      </c>
+      <c r="AV8">
+        <v>7721</v>
+      </c>
+      <c r="AW8">
+        <v>7723</v>
+      </c>
+      <c r="AX8">
+        <v>7730</v>
+      </c>
+      <c r="AY8">
+        <v>7740</v>
+      </c>
+      <c r="AZ8">
+        <v>7785</v>
+      </c>
+      <c r="BA8">
+        <v>8008</v>
+      </c>
+      <c r="BB8">
+        <v>8120</v>
+      </c>
+      <c r="BC8">
+        <v>8217</v>
+      </c>
+      <c r="BD8">
+        <v>8268</v>
+      </c>
+      <c r="BE8">
+        <v>8319</v>
+      </c>
+      <c r="BF8">
+        <v>8343</v>
+      </c>
+      <c r="BG8">
+        <v>8350</v>
+      </c>
+      <c r="BH8">
+        <v>7355</v>
+      </c>
+      <c r="BI8">
+        <v>8442</v>
+      </c>
+      <c r="BJ8">
+        <v>8491</v>
+      </c>
+      <c r="BK8">
+        <v>8839</v>
+      </c>
+      <c r="BL8">
+        <v>8896</v>
+      </c>
+      <c r="BM8">
+        <v>8928</v>
+      </c>
+      <c r="BN8">
+        <v>8978</v>
+      </c>
+      <c r="BO8">
+        <v>8993</v>
+      </c>
+      <c r="BP8">
+        <v>8995</v>
+      </c>
+      <c r="BQ8">
+        <v>8995</v>
+      </c>
+      <c r="BR8">
+        <v>9154</v>
+      </c>
+      <c r="BS8">
+        <v>9196</v>
+      </c>
+      <c r="BT8">
+        <v>9269</v>
+      </c>
+      <c r="BU8">
+        <v>9348</v>
+      </c>
+      <c r="BV8">
+        <v>9406</v>
+      </c>
+      <c r="BW8">
+        <v>9476</v>
+      </c>
+      <c r="BX8">
+        <v>9547</v>
+      </c>
+      <c r="BY8">
+        <v>9585</v>
+      </c>
+      <c r="BZ8">
+        <v>9656</v>
+      </c>
+      <c r="CA8">
+        <v>9881</v>
+      </c>
+      <c r="CB8">
+        <v>9939</v>
+      </c>
+      <c r="CC8">
+        <v>10008</v>
+      </c>
+      <c r="CD8">
+        <v>10120</v>
+      </c>
+      <c r="CE8">
+        <v>10246</v>
+      </c>
+      <c r="CF8">
+        <v>10357</v>
+      </c>
+      <c r="CG8">
+        <v>10499</v>
+      </c>
+      <c r="CH8">
+        <v>10694</v>
+      </c>
+      <c r="CI8">
+        <v>11396</v>
+      </c>
+      <c r="CJ8">
+        <v>11483</v>
+      </c>
+      <c r="CK8">
+        <v>11552</v>
+      </c>
+      <c r="CL8">
+        <v>11553</v>
+      </c>
+    </row>
+    <row r="9" spans="1:90" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>1491</v>
+      </c>
+      <c r="B9">
+        <v>691</v>
+      </c>
+      <c r="C9">
+        <v>1529</v>
+      </c>
+      <c r="D9">
+        <v>2611</v>
+      </c>
+      <c r="E9">
+        <v>3077</v>
+      </c>
+      <c r="F9">
+        <v>3084</v>
+      </c>
+      <c r="G9">
+        <v>3122</v>
+      </c>
+      <c r="H9">
+        <v>3127</v>
+      </c>
+      <c r="I9">
+        <v>3261</v>
+      </c>
+      <c r="J9">
+        <v>3423</v>
+      </c>
+      <c r="K9">
+        <v>3464</v>
+      </c>
+      <c r="L9">
+        <v>3547</v>
+      </c>
+      <c r="M9">
+        <v>3615</v>
+      </c>
+      <c r="N9">
+        <v>3760</v>
+      </c>
+      <c r="O9">
+        <v>3922</v>
+      </c>
+      <c r="P9">
+        <v>4022</v>
+      </c>
+      <c r="Q9">
+        <v>4131</v>
+      </c>
+      <c r="R9">
+        <v>5232</v>
+      </c>
+      <c r="S9">
+        <v>4333</v>
+      </c>
+      <c r="T9">
+        <v>4433</v>
+      </c>
+      <c r="U9">
+        <v>4554</v>
+      </c>
+      <c r="V9">
+        <v>4579</v>
+      </c>
+      <c r="W9">
+        <v>4591</v>
+      </c>
+      <c r="X9">
+        <v>4601</v>
+      </c>
+      <c r="Y9">
+        <v>4607</v>
+      </c>
+      <c r="Z9">
+        <v>4617</v>
+      </c>
+      <c r="AA9">
+        <v>4626</v>
+      </c>
+      <c r="AB9">
+        <v>4626</v>
+      </c>
+      <c r="AC9">
+        <v>4644</v>
+      </c>
+      <c r="AD9">
+        <v>4671</v>
+      </c>
+      <c r="AE9">
+        <v>4731</v>
+      </c>
+      <c r="AF9">
+        <v>4776</v>
+      </c>
+      <c r="AG9">
+        <v>4778</v>
+      </c>
+      <c r="AH9">
+        <v>4780</v>
+      </c>
+      <c r="AI9">
+        <v>4802</v>
+      </c>
+      <c r="AJ9">
+        <v>4803</v>
+      </c>
+      <c r="AK9">
+        <v>4805</v>
+      </c>
+      <c r="AL9">
+        <v>4875</v>
+      </c>
+      <c r="AM9">
+        <v>4977</v>
+      </c>
+      <c r="AN9">
+        <v>5038</v>
+      </c>
+      <c r="AO9">
+        <v>5111</v>
+      </c>
+      <c r="AP9">
+        <v>5166</v>
+      </c>
+      <c r="AQ9">
+        <v>5303</v>
+      </c>
+      <c r="AR9">
+        <v>5538</v>
+      </c>
+      <c r="AS9">
+        <v>5633</v>
+      </c>
+      <c r="AT9">
+        <v>5838</v>
+      </c>
+      <c r="AU9">
+        <v>6275</v>
+      </c>
+      <c r="AV9">
+        <v>6511</v>
+      </c>
+      <c r="AW9">
+        <v>6669</v>
+      </c>
+      <c r="AX9">
+        <v>6697</v>
+      </c>
+      <c r="AY9">
+        <v>6714</v>
+      </c>
+      <c r="AZ9">
+        <v>6735</v>
+      </c>
+      <c r="BA9">
+        <v>6806</v>
+      </c>
+      <c r="BB9">
+        <v>6892</v>
+      </c>
+      <c r="BC9">
+        <v>7005</v>
+      </c>
+      <c r="BD9">
+        <v>7049</v>
+      </c>
+      <c r="BE9">
+        <v>7077</v>
+      </c>
+      <c r="BF9">
+        <v>7101</v>
+      </c>
+      <c r="BG9">
+        <v>7116</v>
+      </c>
+      <c r="BH9">
+        <v>7149</v>
+      </c>
+      <c r="BI9">
+        <v>7321</v>
+      </c>
+      <c r="BJ9">
+        <v>7343</v>
+      </c>
+      <c r="BK9">
+        <v>7609</v>
+      </c>
+      <c r="BL9">
+        <v>7616</v>
+      </c>
+      <c r="BM9">
+        <v>7633</v>
+      </c>
+      <c r="BN9">
+        <v>8174</v>
+      </c>
+      <c r="BO9">
+        <v>8571</v>
+      </c>
+      <c r="BP9">
+        <v>9031</v>
+      </c>
+      <c r="BQ9">
+        <v>9031</v>
+      </c>
+      <c r="BR9">
+        <v>9155</v>
+      </c>
+      <c r="BS9">
+        <v>9243</v>
+      </c>
+      <c r="BT9">
+        <v>9433</v>
+      </c>
+      <c r="BU9">
+        <v>9693</v>
+      </c>
+      <c r="BV9">
+        <v>9912</v>
+      </c>
+      <c r="BW9">
+        <v>10124</v>
+      </c>
+      <c r="BX9">
+        <v>10188</v>
+      </c>
+      <c r="BY9">
+        <v>10227</v>
+      </c>
+      <c r="BZ9">
+        <v>10271</v>
+      </c>
+      <c r="CA9">
+        <v>10414</v>
+      </c>
+      <c r="CB9">
+        <v>10426</v>
+      </c>
+      <c r="CC9">
+        <v>10445</v>
+      </c>
+      <c r="CD9">
+        <v>10473</v>
+      </c>
+      <c r="CE9">
+        <v>10498</v>
+      </c>
+      <c r="CF9">
+        <v>10594</v>
+      </c>
+      <c r="CG9">
+        <v>10617</v>
+      </c>
+      <c r="CH9">
+        <v>10664</v>
+      </c>
+      <c r="CI9">
+        <v>10920</v>
+      </c>
+      <c r="CJ9">
+        <v>10989</v>
+      </c>
+      <c r="CK9">
+        <v>11051</v>
+      </c>
+      <c r="CL9">
+        <v>11052</v>
+      </c>
+    </row>
+    <row r="10" spans="1:90" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>1492</v>
+      </c>
+      <c r="B10">
+        <v>770</v>
+      </c>
+      <c r="C10">
+        <v>1627</v>
+      </c>
+      <c r="D10">
+        <v>2604</v>
+      </c>
+      <c r="E10">
+        <v>3134</v>
+      </c>
+      <c r="F10">
+        <v>3162</v>
+      </c>
+      <c r="G10">
+        <v>3194</v>
+      </c>
+      <c r="H10">
+        <v>3203</v>
+      </c>
+      <c r="I10">
+        <v>3210</v>
+      </c>
+      <c r="J10">
+        <v>3534</v>
+      </c>
+      <c r="K10">
+        <v>3649</v>
+      </c>
+      <c r="L10">
+        <v>3764</v>
+      </c>
+      <c r="M10">
+        <v>3946</v>
+      </c>
+      <c r="N10">
+        <v>4065</v>
+      </c>
+      <c r="O10">
+        <v>4067</v>
+      </c>
+      <c r="P10">
+        <v>4075</v>
+      </c>
+      <c r="Q10">
+        <v>4093</v>
+      </c>
+      <c r="R10">
+        <v>4167</v>
+      </c>
+      <c r="S10">
+        <v>4230</v>
+      </c>
+      <c r="T10">
+        <v>4309</v>
+      </c>
+      <c r="U10">
+        <v>4506</v>
+      </c>
+      <c r="V10">
+        <v>4621</v>
+      </c>
+      <c r="W10">
+        <v>4776</v>
+      </c>
+      <c r="X10">
+        <v>4845</v>
+      </c>
+      <c r="Y10">
+        <v>4931</v>
+      </c>
+      <c r="Z10">
+        <v>5005</v>
+      </c>
+      <c r="AA10">
+        <v>5055</v>
+      </c>
+      <c r="AB10">
+        <v>5055</v>
+      </c>
+      <c r="AC10">
+        <v>5073</v>
+      </c>
+      <c r="AD10">
+        <v>5101</v>
+      </c>
+      <c r="AE10">
+        <v>5182</v>
+      </c>
+      <c r="AF10">
+        <v>5265</v>
+      </c>
+      <c r="AG10">
+        <v>5274</v>
+      </c>
+      <c r="AH10">
+        <v>5291</v>
+      </c>
+      <c r="AI10">
+        <v>5302</v>
+      </c>
+      <c r="AJ10">
+        <v>5303</v>
+      </c>
+      <c r="AK10">
+        <v>5303</v>
+      </c>
+      <c r="AL10">
+        <v>5311</v>
+      </c>
+      <c r="AM10">
+        <v>5451</v>
+      </c>
+      <c r="AN10">
+        <v>5527</v>
+      </c>
+      <c r="AO10">
+        <v>5596</v>
+      </c>
+      <c r="AP10">
+        <v>5708</v>
+      </c>
+      <c r="AQ10">
+        <v>5912</v>
+      </c>
+      <c r="AR10">
+        <v>6177</v>
+      </c>
+      <c r="AS10">
+        <v>6276</v>
+      </c>
+      <c r="AT10">
+        <v>6414</v>
+      </c>
+      <c r="AU10">
+        <v>6452</v>
+      </c>
+      <c r="AV10">
+        <v>6460</v>
+      </c>
+      <c r="AW10">
+        <v>6467</v>
+      </c>
+      <c r="AX10">
+        <v>6495</v>
+      </c>
+      <c r="AY10">
+        <v>6561</v>
+      </c>
+      <c r="AZ10">
+        <v>6674</v>
+      </c>
+      <c r="BA10">
+        <v>6929</v>
+      </c>
+      <c r="BB10">
+        <v>7080</v>
+      </c>
+      <c r="BC10">
+        <v>7220</v>
+      </c>
+      <c r="BD10">
+        <v>7324</v>
+      </c>
+      <c r="BE10">
+        <v>7473</v>
+      </c>
+      <c r="BF10">
+        <v>7552</v>
+      </c>
+      <c r="BG10">
+        <v>7605</v>
+      </c>
+      <c r="BH10">
+        <v>7675</v>
+      </c>
+      <c r="BI10">
+        <v>7917</v>
+      </c>
+      <c r="BJ10">
+        <v>7983</v>
+      </c>
+      <c r="BK10">
+        <v>8624</v>
+      </c>
+      <c r="BL10">
+        <v>8657</v>
+      </c>
+      <c r="BM10">
+        <v>8718</v>
+      </c>
+      <c r="BN10">
+        <v>8759</v>
+      </c>
+      <c r="BO10">
+        <v>8763</v>
+      </c>
+      <c r="BP10">
+        <v>8765</v>
+      </c>
+      <c r="BQ10">
+        <v>8765</v>
+      </c>
+      <c r="BR10">
+        <v>9323</v>
+      </c>
+      <c r="BS10">
+        <v>9423</v>
+      </c>
+      <c r="BT10">
+        <v>9494</v>
+      </c>
+      <c r="BU10">
+        <v>9567</v>
+      </c>
+      <c r="BV10">
+        <v>9667</v>
+      </c>
+      <c r="BW10">
+        <v>9750</v>
+      </c>
+      <c r="BX10">
+        <v>9810</v>
+      </c>
+      <c r="BY10">
+        <v>9885</v>
+      </c>
+      <c r="BZ10">
+        <v>9964</v>
+      </c>
+      <c r="CA10">
+        <v>10222</v>
+      </c>
+      <c r="CB10">
+        <v>10275</v>
+      </c>
+      <c r="CC10">
+        <v>10339</v>
+      </c>
+      <c r="CD10">
+        <v>10423</v>
+      </c>
+      <c r="CE10">
+        <v>10443</v>
+      </c>
+      <c r="CF10">
+        <v>10465</v>
+      </c>
+      <c r="CG10">
+        <v>10534</v>
+      </c>
+      <c r="CH10">
+        <v>10586</v>
+      </c>
+      <c r="CI10">
+        <v>10732</v>
+      </c>
+      <c r="CJ10">
+        <v>10751</v>
+      </c>
+      <c r="CK10">
+        <v>10767</v>
+      </c>
+      <c r="CL10">
+        <v>10767</v>
+      </c>
+    </row>
+    <row r="11" spans="1:90" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>1493</v>
+      </c>
+      <c r="B11">
+        <v>780</v>
+      </c>
+      <c r="C11">
+        <v>1424</v>
+      </c>
+      <c r="D11">
+        <v>2187</v>
+      </c>
+      <c r="E11">
+        <v>2684</v>
+      </c>
+      <c r="F11">
+        <v>2699</v>
+      </c>
+      <c r="G11">
+        <v>2718</v>
+      </c>
+      <c r="H11">
+        <v>2720</v>
+      </c>
+      <c r="I11">
+        <v>2728</v>
+      </c>
+      <c r="J11">
+        <v>2734</v>
+      </c>
+      <c r="K11">
+        <v>2734</v>
+      </c>
+      <c r="L11">
+        <v>2737</v>
+      </c>
+      <c r="M11">
+        <v>2737</v>
+      </c>
+      <c r="N11">
+        <v>2737</v>
+      </c>
+      <c r="O11">
+        <v>2737</v>
+      </c>
+      <c r="P11">
+        <v>2737</v>
+      </c>
+      <c r="Q11">
+        <v>2737</v>
+      </c>
+      <c r="R11">
+        <v>2737</v>
+      </c>
+      <c r="S11">
+        <v>2739</v>
+      </c>
+      <c r="T11">
+        <v>2739</v>
+      </c>
+      <c r="U11">
+        <v>2740</v>
+      </c>
+      <c r="V11">
+        <v>2740</v>
+      </c>
+      <c r="W11">
+        <v>2740</v>
+      </c>
+      <c r="X11">
+        <v>2740</v>
+      </c>
+      <c r="Y11">
+        <v>2740</v>
+      </c>
+      <c r="Z11">
+        <v>2740</v>
+      </c>
+      <c r="AA11">
+        <v>2740</v>
+      </c>
+      <c r="AB11">
+        <v>2740</v>
+      </c>
+      <c r="AC11">
+        <v>2740</v>
+      </c>
+      <c r="AD11">
+        <v>2740</v>
+      </c>
+      <c r="AE11">
+        <v>2740</v>
+      </c>
+      <c r="AF11">
+        <v>2740</v>
+      </c>
+      <c r="AG11">
+        <v>2740</v>
+      </c>
+      <c r="AH11">
+        <v>2741</v>
+      </c>
+      <c r="AI11">
+        <v>2742</v>
+      </c>
+      <c r="AJ11">
+        <v>2742</v>
+      </c>
+      <c r="AK11">
+        <v>2742</v>
+      </c>
+      <c r="AL11">
+        <v>2742</v>
+      </c>
+      <c r="AM11">
+        <v>2742</v>
+      </c>
+      <c r="AN11">
+        <v>2742</v>
+      </c>
+      <c r="AO11">
+        <v>2742</v>
+      </c>
+      <c r="AP11">
+        <v>2742</v>
+      </c>
+      <c r="AQ11">
+        <v>2742</v>
+      </c>
+      <c r="AR11">
+        <v>2742</v>
+      </c>
+      <c r="AS11">
+        <v>2742</v>
+      </c>
+      <c r="AT11">
+        <v>2742</v>
+      </c>
+      <c r="AU11">
+        <v>2743</v>
+      </c>
+      <c r="AV11">
+        <v>2749</v>
+      </c>
+      <c r="AW11">
+        <v>2753</v>
+      </c>
+      <c r="AX11">
+        <v>2758</v>
+      </c>
+      <c r="AY11">
+        <v>2768</v>
+      </c>
+      <c r="AZ11">
+        <v>2769</v>
+      </c>
+      <c r="BA11">
+        <v>2769</v>
+      </c>
+      <c r="BB11">
+        <v>2770</v>
+      </c>
+      <c r="BC11">
+        <v>2770</v>
+      </c>
+      <c r="BD11">
+        <v>2770</v>
+      </c>
+      <c r="BE11">
+        <v>2770</v>
+      </c>
+      <c r="BF11">
+        <v>2770</v>
+      </c>
+      <c r="BG11">
+        <v>2770</v>
+      </c>
+      <c r="BH11">
+        <v>2771</v>
+      </c>
+      <c r="BI11">
+        <v>2771</v>
+      </c>
+      <c r="BJ11">
+        <v>2771</v>
+      </c>
+      <c r="BK11">
+        <v>2777</v>
+      </c>
+      <c r="BL11">
+        <v>2777</v>
+      </c>
+      <c r="BM11">
+        <v>2778</v>
+      </c>
+      <c r="BN11">
+        <v>2781</v>
+      </c>
+      <c r="BO11">
+        <v>2781</v>
+      </c>
+      <c r="BP11">
+        <v>2782</v>
+      </c>
+      <c r="BQ11">
+        <v>2785</v>
+      </c>
+      <c r="BR11">
+        <v>2796</v>
+      </c>
+      <c r="BS11">
+        <v>2796</v>
+      </c>
+      <c r="BT11">
+        <v>2796</v>
+      </c>
+      <c r="BU11">
+        <v>2796</v>
+      </c>
+      <c r="BV11">
+        <v>2797</v>
+      </c>
+      <c r="BW11">
+        <v>2797</v>
+      </c>
+      <c r="BX11">
+        <v>2797</v>
+      </c>
+      <c r="BY11">
+        <v>2797</v>
+      </c>
+      <c r="BZ11">
+        <v>2797</v>
+      </c>
+      <c r="CA11">
+        <v>2797</v>
+      </c>
+      <c r="CB11">
+        <v>2797</v>
+      </c>
+      <c r="CC11">
+        <v>2797</v>
+      </c>
+      <c r="CD11">
+        <v>2797</v>
+      </c>
+      <c r="CE11">
+        <v>2797</v>
+      </c>
+      <c r="CF11">
+        <v>2797</v>
+      </c>
+      <c r="CG11">
+        <v>2798</v>
+      </c>
+      <c r="CH11">
+        <v>2799</v>
+      </c>
+      <c r="CI11">
+        <v>2799</v>
+      </c>
+      <c r="CJ11">
+        <v>2799</v>
+      </c>
+      <c r="CK11">
+        <v>2799</v>
+      </c>
+      <c r="CL11">
+        <v>2799</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>